<commit_message>
Add pooled n=6 analysis and update Source Data
- analysis/ses_pooled_n6_corr_20260820.py: analyses with all six
  participants treated as a single group (protocol version not used as a
  factor), including the descriptive Pearson correlation reported in
  Figure S7 and the leave-one-out coefficients.
- analysis/make_supp_fig_S7_20260820.py: script that draws Figure S7.
- data/Source_Data_1.xlsx: adds the FigS7_Pooled sheet; removes the ten
  between-version p-values that remained in the Fig5 and FigS4 sheets, so
  that the file matches its own statement that no inferential statistic is
  reported anywhere in it.
</commit_message>
<xml_diff>
--- a/data/Source_Data_1.xlsx
+++ b/data/Source_Data_1.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6b_CrossClassification" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6c_IntensityBands" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig6d_Bouts_sound_vs_nosound" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS7_Pooled" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -512,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,7 +629,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes - between-version p-values removed (R1-6)</t>
         </is>
       </c>
     </row>
@@ -781,7 +782,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes - between-version p-values removed (R1-6)</t>
         </is>
       </c>
     </row>
@@ -839,6 +840,23 @@
     <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t>FigS7_Pooled</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Figure S7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>yes - new</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>No inferential statistic is reported anywhere in this file. Where a correlation coefficient appears it is descriptive and no p-value accompanies it.</t>
         </is>
@@ -868,7 +886,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="21">
       <c r="A3" s="11" t="inlineStr">
         <is>
@@ -1006,8 +1023,6 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="21">
       <c r="A13" s="11" t="inlineStr">
         <is>
@@ -1650,14 +1665,8 @@
           <t>-8.5 [-22.3 to 5.3]</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="n">
-        <v>0.151</v>
-      </c>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="21">
       <c r="A13" s="10" t="inlineStr">
@@ -1675,14 +1684,8 @@
           <t>-2.5 [-5.8 to 0.8]</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>0.106</v>
-      </c>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="21">
       <c r="A14" s="10" t="inlineStr">
@@ -1700,14 +1703,8 @@
           <t>-1.8 [-5.0 to 1.5]</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="n">
-        <v>0.188</v>
-      </c>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="21">
       <c r="A15" s="10" t="inlineStr">
@@ -1725,14 +1722,8 @@
           <t>-4.3 [-11.0 to 2.5]</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="n">
-        <v>0.145</v>
-      </c>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="10" t="inlineStr">
@@ -1750,14 +1741,8 @@
           <t>0.0 [-2.9 to 2.9]</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="n">
-        <v>1</v>
-      </c>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1787,7 +1772,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="21">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2217,7 +2201,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="21">
       <c r="A11" s="9" t="inlineStr">
         <is>
@@ -2233,7 +2216,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.83 [-5.72 to 7.38], p=0.757</t>
+          <t>0.83 [-5.72 to 7.38]</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2228,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>-1.17 [-8.11 to 5.78], p=0.684</t>
+          <t>-1.17 [-8.11 to 5.78]</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2240,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>-0.8 [-2.6 to 1.0], p=0.289</t>
+          <t>-0.8 [-2.6 to 1.0]</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2252,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-1.3 [-3.3 to 0.6], p=0.140</t>
+          <t>-1.3 [-3.3 to 0.6]</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2264,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>-0.3 [-2.8 to 2.1], p=0.741</t>
+          <t>-0.3 [-2.8 to 2.1]</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2300,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -2621,7 +2603,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2844,7 +2825,6 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -2873,7 +2853,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3147,7 +3126,6 @@
         <v>146</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3176,7 +3154,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3424,11 +3401,10 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Note. The advancing-window criterion is the rule the device applied in real time and is the one that produces Table 2 (a 30-s window advancing in 1-s steps, at least 6 s of slow-wave activity, seconds overlapping a marked arousal excluded). The technologist's scoring uses the fixed clock-aligned 30-s grid and produces Figure 6b. Of the 519 s that met the advancing-window criterion alone, 497 s were scored N2 and 22 s wake by the technologist.</t>
+          <t>Note. The advancing-window criterion is applied post hoc to the delivered seconds and is the one that produces Table 2. It is not the rule that gated playback: playback began after three consecutive 30-s epochs in each of which at least 90% of the preceding 30 s had been marked as slow-wave sleep by the technologist, and stopped when the technologist judged that slow-wave sleep had been interrupted (Methods) (a 30-s window advancing in 1-s steps, at least 6 s of slow-wave activity, seconds overlapping a marked arousal excluded). The technologist's scoring uses the fixed clock-aligned 30-s grid and produces Figure 6b. Of the 519 s that met the advancing-window criterion alone, 497 s were scored N2 and 22 s wake by the technologist.</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3436,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3902,7 +3877,6 @@
         <v>62.3</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3931,7 +3905,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4151,11 +4124,309 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>Note. Sound begins only after 90 s of sustained slow-wave sleep and stops at a cumulative 600 s, so most slow-wave sleep on the SES night carried no sound. Between zero and five bouts of at least 90 s contained sound in each participant (H14 had none), so no comparison is made against that column.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" style="21" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Figure S7. Pooled association between change in SUDS and change in PCL-5 intrusion (all six participants; version not used as a factor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Participant</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pre-SES SUDS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Post-SES SUDS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SUDS change % ((post-pre)/pre x100)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PCL-5 intrusion Pre</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PCL-5 intrusion FU</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PCL-5 intrusion Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>H01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>30</v>
+      </c>
+      <c r="D3" t="n">
+        <v>35</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>H02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>35</v>
+      </c>
+      <c r="D4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E4" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>H03</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D5" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-50</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>H08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-50</v>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>H09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-80</v>
+      </c>
+      <c r="F7" t="n">
+        <v>14</v>
+      </c>
+      <c r="G7" t="n">
+        <v>7</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>H14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Pearson r (SUDS change % vs PCL-5 intrusion change), n = 6</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Range of r across the six leave-one-out analyses</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>+0.94 to +0.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Pearson r among the four amended-version participants only</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Note. Descriptive coefficient. No significance testing was performed and no p-value is reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pooled paired change, SUDS (points): mean -13.3, SD 18.4, 95% CI -32.6 to +5.9, Cohen's dz -0.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Pooled paired change, PCL-5 intrusion (points): mean -2.7, SD 4.1, 95% CI -7.0 to +1.7, Cohen's dz -0.65</t>
         </is>
       </c>
     </row>
@@ -4190,7 +4461,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="39.5" customHeight="1" s="21">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -4764,7 +5034,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="21">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -9198,7 +9467,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="21">
       <c r="A3" t="inlineStr">
         <is>
@@ -9368,7 +9636,6 @@
         <v>68.2</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -9418,7 +9685,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26.25" customHeight="1" s="21">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -9630,7 +9896,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="21">
       <c r="A11" s="9" t="inlineStr">
         <is>
@@ -9664,14 +9929,7 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="21">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>P value</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>0.0124</v>
-      </c>
+      <c r="A14" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10155,14 +10413,8 @@
           <t>-14.0 [-30.4 to 2.4]</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="n">
-        <v>0.073</v>
-      </c>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="21">
       <c r="A13" s="10" t="inlineStr">
@@ -10180,14 +10432,8 @@
           <t>-7.0 [-11.6 to -2.4]</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>0.015</v>
-      </c>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="21">
       <c r="A14" s="10" t="inlineStr">
@@ -10205,14 +10451,8 @@
           <t>-2.5 [-5.5 to 0.5]</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="n">
-        <v>0.08</v>
-      </c>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="21">
       <c r="A15" s="10" t="inlineStr">
@@ -10230,14 +10470,8 @@
           <t>-3.5 [-11.3 to 4.3]</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="n">
-        <v>0.278</v>
-      </c>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="21">
       <c r="A16" s="10" t="inlineStr">
@@ -10255,14 +10489,8 @@
           <t>-1.0 [-7.8 to 5.8]</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="E16" s="10" t="n">
-        <v>0.67</v>
-      </c>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10292,7 +10520,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28.5" customHeight="1" s="21">
       <c r="A3" t="inlineStr">
         <is>
@@ -10465,7 +10692,6 @@
         <v>-2.7273</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -10503,7 +10729,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -10545,7 +10770,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="28.5" customHeight="1" s="21">
       <c r="A3" t="inlineStr">
         <is>
@@ -10699,7 +10923,6 @@
         <v>29.78</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -10750,7 +10973,6 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -10792,7 +11014,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="26.25" customHeight="1" s="21">
       <c r="A3" t="inlineStr">
         <is>
@@ -10923,7 +11144,6 @@
         <v>-0.2</v>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="21">
       <c r="A11" t="inlineStr">
         <is>

</xml_diff>